<commit_message>
Add turtle to map, PK in schema
</commit_message>
<xml_diff>
--- a/Rekindle the Green Database Schema.xlsx
+++ b/Rekindle the Green Database Schema.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a7b2e265512bf4b7/Documents/college/WPL/WildLink/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a7b2e265512bf4b7/Documents/college/WPL/Rekindle-the-Green/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8627C4DC-4674-4145-A004-EDBF6CB81C42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{8627C4DC-4674-4145-A004-EDBF6CB81C42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE619E39-EEF6-4665-A7AF-81BC3B453FC1}"/>
   <bookViews>
     <workbookView xWindow="528" yWindow="792" windowWidth="19404" windowHeight="10740" xr2:uid="{E049C550-504B-4D65-B260-6756B5056B05}"/>
   </bookViews>
@@ -78,8 +78,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -122,9 +130,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -468,7 +477,7 @@
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -490,7 +499,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="1" t="s">

</xml_diff>